<commit_message>
docs: automation complete — 190 tasks, web interface verified
- Update GATEKEEPER_STATUS.md: mark all seeding steps complete,
  restructure Next Actions into Completed Steps + Future Actions
- Add .gitignore rules for __pycache__, *.pyc, Thumbs.db, ~$ temp files
- Add extracted reference docs (SIA WHS BOK, Singleton Council)
  replacing zip archives
- Add new source files: compress_swms.py, swms_to_html.py
- Add generated outputs: Crack Stitching, Render Patching,
  Scaffold Erection, Painting SWMS
- Remove old Master SWMS .docx outputs (superseded by DB-driven generation)
- Web interface tested: /health, /tasks (190), index page all OK

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rpd-v8-upgrade/phase-2-whsmp-update/swms/RPD_SWMS_Consolidation_Traceability_Map_1.xlsx
+++ b/rpd-v8-upgrade/phase-2-whsmp-update/swms/RPD_SWMS_Consolidation_Traceability_Map_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlanRichardson\gatekeeper\rpd-v8-upgrade\phase-2-whsmp-update\swms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB388C3-81F9-4696-B775-7FF4632DCF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E17C2FE8-2A75-4FB9-A4B9-E4C6C02462EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30435" yWindow="-3645" windowWidth="20070" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29280" yWindow="-3645" windowWidth="20745" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="New SWMS Structure" sheetId="2" r:id="rId1"/>
@@ -669,7 +669,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -704,6 +704,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -840,6 +846,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -848,19 +864,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1177,22 +1187,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
     </row>
     <row r="4" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1232,16 +1242,16 @@
       <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="21" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1249,16 +1259,16 @@
       <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="21" t="s">
         <v>150</v>
       </c>
     </row>
@@ -1490,7 +1500,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="24" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="36" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
         <v>192</v>
       </c>
@@ -1504,7 +1514,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="75" fitToWidth="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1527,40 +1537,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1589,16 +1599,16 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
@@ -1883,22 +1893,22 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10">
+      <c r="A18" s="16">
         <v>12</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="12"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="18"/>
     </row>
     <row r="19" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="18"/>
+      <c r="B19" s="15"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>

</xml_diff>